<commit_message>
New changes in materials and volumetry
</commit_message>
<xml_diff>
--- a/src/assets/documents/FORMATO_MATERIALES.xlsx
+++ b/src/assets/documents/FORMATO_MATERIALES.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aemo/Projects/bellarti-app/src/assets/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11B5E881-5A51-E04E-B85F-AE2CD5F728B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{386FF325-A588-1549-A618-600CD2EA6DD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-51200" yWindow="0" windowWidth="51200" windowHeight="28800" xr2:uid="{C1CA46D1-D146-E345-A83F-B7A5E76EA8D7}"/>
+    <workbookView xWindow="-51200" yWindow="620" windowWidth="51200" windowHeight="28180" xr2:uid="{C1CA46D1-D146-E345-A83F-B7A5E76EA8D7}"/>
   </bookViews>
   <sheets>
     <sheet name="MATERIALES" sheetId="1" r:id="rId1"/>
@@ -114,9 +114,6 @@
     <t>DIVISIÓN</t>
   </si>
   <si>
-    <t>MATERIAL SKU</t>
-  </si>
-  <si>
     <t>ESPEC.1 SKU</t>
   </si>
   <si>
@@ -211,6 +208,9 @@
   </si>
   <si>
     <t>TUBO</t>
+  </si>
+  <si>
+    <t>MATERIAL</t>
   </si>
 </sst>
 </file>
@@ -282,345 +282,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="14">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9A9FF"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFC000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFA8"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="5" tint="-0.24994659260841701"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC2C3"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7773"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF0070C0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFA7FCFF"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF676FF"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF0070C0"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -934,7 +596,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="5" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="19.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18.6640625" bestFit="1" customWidth="1"/>
@@ -956,22 +618,22 @@
         <v>24</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>30</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>0</v>
@@ -1007,7 +669,7 @@
         <v>23</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1069,21 +731,21 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
@@ -1092,12 +754,12 @@
         <v>2</v>
       </c>
       <c r="D2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
@@ -1106,12 +768,12 @@
         <v>3</v>
       </c>
       <c r="D3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s">
         <v>6</v>
@@ -1119,7 +781,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B5" t="s">
         <v>7</v>
@@ -1127,7 +789,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
@@ -1135,7 +797,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B7" t="s">
         <v>13</v>
@@ -1143,7 +805,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B8" t="s">
         <v>9</v>
@@ -1151,7 +813,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B9" t="s">
         <v>14</v>
@@ -1159,7 +821,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B10" t="s">
         <v>10</v>
@@ -1167,7 +829,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B11" t="s">
         <v>11</v>
@@ -1175,7 +837,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B12" t="s">
         <v>12</v>
@@ -1183,39 +845,39 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B15" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>